<commit_message>
Set party hours 17h-3h30, make the intro wave cut into the hero photo
The cream band under the hero was the wave itself: it sat at the top of
the intro filled with the page background, so against a photo it read as
an empty strip. Moves it to the bottom of the hero filled with the intro
gradient's first colour instead, so the blue wave rises into the photo
and meets the intro seamlessly.

The calendar link also mixed time bases — the start was formatted from
local wall-clock while the end went through toISOString(), i.e. UTC, so
the event ran two hours short. Both ends are now explicit config values
with ctz=Europe/Paris, and the venue address is included in the invite.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -117,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +132,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -663,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -689,12 +692,12 @@
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>P01</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Noms du couple</t>
         </is>
@@ -706,12 +709,12 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>P02</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Date affichée</t>
         </is>
@@ -723,115 +726,132 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>P03</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Date + heure réelle (agenda)</t>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Début de l'événement (agenda)</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>2027-04-24T16:30:00</t>
+          <t>2027-04-24T17:00:00</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>P04</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Fin de l'événement (agenda)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>2027-04-25T03:30:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Nom du lieu</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>La Ferme de la Faisanderie</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>P05</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Adresse du lieu</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Route de Rennemoulin, 78450 Villepreux</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Recherche Google Maps</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Ferme de la Faisanderie, Route de Rennemoulin, 78450 Villepreux</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>P07</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Date limite de réponse</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>1er mai 2026</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>P08</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Lien du formulaire RSVP</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>P09</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Lien de la cagnotte</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr"/>
+      <c r="C11" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -879,12 +899,12 @@
       <c r="C2" s="7" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>A01</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -896,12 +916,12 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>A02</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Noms</t>
         </is>
@@ -913,12 +933,12 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>A03</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -930,12 +950,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>A04</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Lieu</t>
         </is>
@@ -947,12 +967,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>A05</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Invitation à défiler</t>
         </is>
@@ -973,12 +993,12 @@
       <c r="C8" s="7" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>A06</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Paragraphe</t>
         </is>
@@ -990,12 +1010,12 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>A07</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -1016,12 +1036,12 @@
       <c r="C11" s="7" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>A08</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1033,12 +1053,12 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>A09</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1050,12 +1070,12 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>A10</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -1067,12 +1087,12 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>A11</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Étiquette 1</t>
         </is>
@@ -1084,12 +1104,12 @@
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>A12</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Étiquette 2</t>
         </is>
@@ -1101,12 +1121,12 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>A13</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Étiquette 3</t>
         </is>
@@ -1118,12 +1138,12 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>A14</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Étiquette 4</t>
         </is>
@@ -1135,12 +1155,12 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>A15</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Lien agenda</t>
         </is>
@@ -1161,12 +1181,12 @@
       <c r="C20" s="7" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>A16</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1178,12 +1198,12 @@
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>A17</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1195,12 +1215,12 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>A18</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Carte 1 — titre</t>
         </is>
@@ -1212,12 +1232,12 @@
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>A19</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Carte 1 — lien</t>
         </is>
@@ -1229,12 +1249,12 @@
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>A20</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Carte 2 — titre</t>
         </is>
@@ -1246,12 +1266,12 @@
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>A21</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Carte 2 — texte</t>
         </is>
@@ -1263,12 +1283,12 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>A22</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Carte 3 — titre</t>
         </is>
@@ -1280,12 +1300,12 @@
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>A23</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Carte 3 — texte</t>
         </is>
@@ -1297,12 +1317,12 @@
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>A24</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Carte 4 — titre</t>
         </is>
@@ -1314,12 +1334,12 @@
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>A25</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Carte 4 — texte</t>
         </is>
@@ -1340,12 +1360,12 @@
       <c r="C31" s="7" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>A26</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1357,12 +1377,12 @@
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>A27</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1374,12 +1394,12 @@
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>A28</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Texte</t>
         </is>
@@ -1391,12 +1411,12 @@
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>A29</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -1408,19 +1428,19 @@
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>Date limite</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Merci de répondre avant le [date — voir P07]</t>
+          <t>Merci de répondre avant le [date — voir onglet Paramètres (P08)]</t>
         </is>
       </c>
     </row>
@@ -1434,12 +1454,12 @@
       <c r="C37" s="7" t="n"/>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>A31</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1451,12 +1471,12 @@
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>A32</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1468,12 +1488,12 @@
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>A33</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>Texte</t>
         </is>
@@ -1485,12 +1505,12 @@
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>A34</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -1511,12 +1531,12 @@
       <c r="C42" s="7" t="n"/>
     </row>
     <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>A35</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B43" s="8" t="inlineStr">
         <is>
           <t>Signature</t>
         </is>
@@ -1528,12 +1548,12 @@
       </c>
     </row>
     <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>A36</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>Petite phrase</t>
         </is>
@@ -1545,12 +1565,12 @@
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>A37</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B45" s="8" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -1571,12 +1591,12 @@
       <c r="C46" s="7" t="n"/>
     </row>
     <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>A38</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B47" s="8" t="inlineStr">
         <is>
           <t>Titre de l'onglet</t>
         </is>
@@ -1588,12 +1608,12 @@
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>A39</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>Description au partage</t>
         </is>
@@ -1650,12 +1670,12 @@
       <c r="C2" s="7" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>H01</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Lien retour</t>
         </is>
@@ -1667,12 +1687,12 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>H02</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Lien raccourci</t>
         </is>
@@ -1693,12 +1713,12 @@
       <c r="C5" s="7" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>H03</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1710,12 +1730,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>H04</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1727,12 +1747,12 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>H05</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -1753,12 +1773,12 @@
       <c r="C9" s="7" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>H06</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -1770,12 +1790,12 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>H07</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1787,12 +1807,12 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>H08</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -1804,12 +1824,12 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>H09</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Étiquette album 1</t>
         </is>
@@ -1821,12 +1841,12 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>H10</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Étiquette album 2</t>
         </is>
@@ -1847,12 +1867,12 @@
       <c r="C15" s="7" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>H11</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -1864,12 +1884,12 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>H12</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1881,12 +1901,12 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>H13</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -1898,12 +1918,12 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>H14</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Étiquette album 1</t>
         </is>
@@ -1915,12 +1935,12 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>H15</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Étiquette album 2</t>
         </is>
@@ -1941,12 +1961,12 @@
       <c r="C21" s="7" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>H16</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -1958,12 +1978,12 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>H17</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1975,12 +1995,12 @@
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>H18</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -2001,12 +2021,12 @@
       <c r="C25" s="7" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>H19</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -2018,12 +2038,12 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>H20</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Phrase de fin</t>
         </is>
@@ -2035,12 +2055,12 @@
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>H21</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Texte</t>
         </is>
@@ -2052,12 +2072,12 @@
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>H22</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -2078,12 +2098,12 @@
       <c r="C30" s="7" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>H23</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Titre de l'onglet</t>
         </is>
@@ -2095,12 +2115,12 @@
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>H24</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Description au partage</t>
         </is>
@@ -2171,12 +2191,12 @@
       <c r="E2" s="7" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>F01</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Ouverture</t>
         </is>
@@ -2184,7 +2204,7 @@
       <c r="C3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>histoire-01-ouverture.jpg</t>
         </is>
@@ -2207,12 +2227,12 @@
       <c r="E4" s="7" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>F02</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2220,7 +2240,7 @@
       <c r="C5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-1.jpg</t>
         </is>
@@ -2232,12 +2252,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>F03</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2245,7 +2265,7 @@
       <c r="C6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-2.jpg</t>
         </is>
@@ -2257,12 +2277,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>F04</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2270,7 +2290,7 @@
       <c r="C7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-3.jpg</t>
         </is>
@@ -2282,12 +2302,12 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>F05</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2295,7 +2315,7 @@
       <c r="C8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-4.jpg</t>
         </is>
@@ -2307,12 +2327,12 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>F06</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2320,7 +2340,7 @@
       <c r="C9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-5.jpg</t>
         </is>
@@ -2332,12 +2352,12 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>F07</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2345,7 +2365,7 @@
       <c r="C10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-6.jpg</t>
         </is>
@@ -2368,12 +2388,12 @@
       <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>F08</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -2381,7 +2401,7 @@
       <c r="C12" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-1.jpg</t>
         </is>
@@ -2393,12 +2413,12 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>F09</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -2406,7 +2426,7 @@
       <c r="C13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-2.jpg</t>
         </is>
@@ -2418,12 +2438,12 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>F10</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -2431,7 +2451,7 @@
       <c r="C14" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-3.jpg</t>
         </is>
@@ -2443,12 +2463,12 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>F11</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -2456,7 +2476,7 @@
       <c r="C15" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-4.jpg</t>
         </is>
@@ -2479,12 +2499,12 @@
       <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>F12</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -2492,7 +2512,7 @@
       <c r="C17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-1.jpg</t>
         </is>
@@ -2504,12 +2524,12 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>F13</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -2517,7 +2537,7 @@
       <c r="C18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-2.jpg</t>
         </is>
@@ -2529,12 +2549,12 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>F14</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -2542,7 +2562,7 @@
       <c r="C19" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-3.jpg</t>
         </is>
@@ -2554,12 +2574,12 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>F15</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -2567,7 +2587,7 @@
       <c r="C20" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-4.jpg</t>
         </is>
@@ -2579,12 +2599,12 @@
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>F16</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -2592,7 +2612,7 @@
       <c r="C21" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-5.jpg</t>
         </is>
@@ -2604,12 +2624,12 @@
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>F17</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -2617,7 +2637,7 @@
       <c r="C22" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-6.jpg</t>
         </is>
@@ -2640,12 +2660,12 @@
       <c r="E23" s="7" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>F18</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -2653,7 +2673,7 @@
       <c r="C24" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-1.jpg</t>
         </is>
@@ -2665,12 +2685,12 @@
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>F19</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -2678,7 +2698,7 @@
       <c r="C25" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-2.jpg</t>
         </is>
@@ -2690,12 +2710,12 @@
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>F20</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -2703,7 +2723,7 @@
       <c r="C26" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-3.jpg</t>
         </is>
@@ -2715,12 +2735,12 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>F21</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -2728,7 +2748,7 @@
       <c r="C27" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-4.jpg</t>
         </is>
@@ -2740,12 +2760,12 @@
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>F22</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -2753,7 +2773,7 @@
       <c r="C28" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-5.jpg</t>
         </is>
@@ -2765,12 +2785,12 @@
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>F23</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -2778,7 +2798,7 @@
       <c r="C29" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-6.jpg</t>
         </is>
@@ -2801,12 +2821,12 @@
       <c r="E30" s="7" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>F24</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -2814,7 +2834,7 @@
       <c r="C31" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-1.jpg</t>
         </is>
@@ -2822,12 +2842,12 @@
       <c r="E31" s="6" t="inlineStr"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>F25</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -2835,7 +2855,7 @@
       <c r="C32" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D32" s="8" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-2.jpg</t>
         </is>
@@ -2843,12 +2863,12 @@
       <c r="E32" s="6" t="inlineStr"/>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>F26</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -2856,7 +2876,7 @@
       <c r="C33" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-3.jpg</t>
         </is>
@@ -2864,12 +2884,12 @@
       <c r="E33" s="6" t="inlineStr"/>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>F27</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -2877,7 +2897,7 @@
       <c r="C34" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-4.jpg</t>
         </is>
@@ -2885,12 +2905,12 @@
       <c r="E34" s="6" t="inlineStr"/>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>F28</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -2898,7 +2918,7 @@
       <c r="C35" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-5.jpg</t>
         </is>
@@ -2917,12 +2937,12 @@
       <c r="E36" s="7" t="n"/>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>F29</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>Épilogue</t>
         </is>
@@ -2930,7 +2950,7 @@
       <c r="C37" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>histoire-07-epilogue.jpg</t>
         </is>

</xml_diff>

<commit_message>
Add an accommodation section to the practical info
Ten places taken from the couple's printed guest sheet, split the way it
groups them: gîtes and houses as cards with their distance and blurb,
hotels as a compact list since the sheet gives them no description.

Adds a matching nav dot, and a Hébergements tab in textes-site.xlsx so
places can be added, reordered or removed without touching the HTML.

La Ferme de Mezu has no URL on the sheet (it says "Réservation sur Gîtes
de France"), so it is listed without a link rather than guessing one.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Mode d'emploi" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Paramètres" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Accueil" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Histoire - textes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Histoire - photos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Hébergements" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Histoire - textes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Histoire - photos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -117,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -133,6 +134,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -500,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B25"/>
+  <dimension ref="B2:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -652,6 +659,34 @@
       <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Videz simplement la cellule (c'est le cas du chapitre III aujourd'hui).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Ajouter ou retirer un hébergement</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Dans l'onglet « Hébergements », ajoutez une ligne (laissez l'ID vide, je le remplirai)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>ou écrivez SUPPRIMER dans la colonne « Ordre ». Le groupe « Hôtels » n'affiche pas</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>les descriptions sur le site : seuls le nom et le lien sont repris.</t>
         </is>
       </c>
     </row>
@@ -864,7 +899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1353,122 +1388,122 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>RÉPONSE (RSVP)</t>
+          <t>HÉBERGEMENTS</t>
         </is>
       </c>
       <c r="B31" s="7" t="n"/>
       <c r="C31" s="7" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>A26</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Votre réponse</t>
+          <t>Où dormir</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>A27</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Serez-vous des nôtres ?</t>
+          <t>Hébergements</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>A28</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>Texte</t>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Texte d'introduction</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Un petit clic pour nous confirmer votre présence (et celle de vos éventuels accompagnants) — ça nous aide énormément pour l'organisation.</t>
+          <t>Quelques adresses repérées autour de la ferme. Pensez à réserver tôt, le printemps est une saison très demandée dans le coin.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>A29</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Bouton</t>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Titre du groupe 1</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Je confirme ma présence</t>
+          <t>Gîtes et maisons</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>Date limite</t>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Titre du groupe 2</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Merci de répondre avant le [date — voir onglet Paramètres (P08)]</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>CAGNOTTE</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="n"/>
-      <c r="C37" s="7" t="n"/>
+          <t>Hôtels</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>A31</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Sous-titre groupe 2</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Un peu plus éloigné — environ 10 min en voiture</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>A31</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>Surtitre</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>Pour nous gâter</t>
-        </is>
-      </c>
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>RÉPONSE (RSVP)</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n"/>
+      <c r="C38" s="7" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
@@ -1478,12 +1513,12 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Titre</t>
+          <t>Surtitre</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Une cagnotte plutôt que des cadeaux</t>
+          <t>Votre réponse</t>
         </is>
       </c>
     </row>
@@ -1495,12 +1530,12 @@
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Texte</t>
+          <t>Titre</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Votre présence est le plus beau des cadeaux. Si vous souhaitez tout de même nous offrir quelque chose, une petite cagnotte est ouverte — sans aucune obligation.</t>
+          <t>Serez-vous des nôtres ?</t>
         </is>
       </c>
     </row>
@@ -1512,57 +1547,57 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
+          <t>Texte</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Un petit clic pour nous confirmer votre présence (et celle de vos éventuels accompagnants) — ça nous aide énormément pour l'organisation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>A35</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
           <t>Bouton</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>Accéder à la cagnotte</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>PIED DE PAGE</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="n"/>
-      <c r="C42" s="7" t="n"/>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Je confirme ma présence</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>A35</t>
+          <t>A36</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Signature</t>
+          <t>Date limite</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>→ voir onglet Paramètres (P01)</t>
+          <t>Merci de répondre avant le [date — voir onglet Paramètres (P08)]</t>
         </is>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>A36</t>
-        </is>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>Petite phrase</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>Avec impatience de vous voir tous réunis.</t>
-        </is>
-      </c>
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>CAGNOTTE</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n"/>
+      <c r="C44" s="7" t="n"/>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
@@ -1572,53 +1607,164 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Bouton</t>
+          <t>Surtitre</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Notre histoire →</t>
+          <t>Pour nous gâter</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>PARTAGE (aperçu WhatsApp / réseaux)</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="n"/>
-      <c r="C46" s="7" t="n"/>
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>A38</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Titre</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Une cagnotte plutôt que des cadeaux</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>A38</t>
+          <t>A39</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Titre de l'onglet</t>
+          <t>Texte</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Awéna &amp; Grégoire — 24 avril 2027</t>
+          <t>Votre présence est le plus beau des cadeaux. Si vous souhaitez tout de même nous offrir quelque chose, une petite cagnotte est ouverte — sans aucune obligation.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>A39</t>
+          <t>A40</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
+          <t>Bouton</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Accéder à la cagnotte</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>PIED DE PAGE</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n"/>
+      <c r="C49" s="7" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>A41</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>→ voir onglet Paramètres (P01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>A42</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Petite phrase</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Avec impatience de vous voir tous réunis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>A43</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>Bouton</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Notre histoire →</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>PARTAGE (aperçu WhatsApp / réseaux)</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="n"/>
+      <c r="C53" s="7" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>A44</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>Titre de l'onglet</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Awéna &amp; Grégoire — 24 avril 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>A45</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
           <t>Description au partage</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>On se marie à la Ferme de la Faisanderie. On serait ravis de vous avoir à nos côtés.</t>
         </is>
@@ -1630,6 +1776,386 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Groupe</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Ordre</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Lien</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>GÎTES ET MAISONS</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Gîtes et maisons</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Le Gîte de la Ferme de Pontaly</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>À 10 min</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Une véritable ferme agricole spécialisée en grandes cultures bio. Elle possède 3 gîtes, de 4 à 8 personnes.</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>https://www.fermedepontaly.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>L02</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Gîtes et maisons</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>La Ferme de Mezu</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>À 5 min</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Jolie ferme équestre et céréalière à Chavenay, en plein milieu des champs. 2 gîtes ruraux (4 et 6 personnes). Réservation sur Gîtes de France.</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr"/>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>L03</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Gîtes et maisons</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Le Val Trebbia</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Maison d'hôtes située à Feucherolles.</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>https://val-trebbia.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>L04</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Gîtes et maisons</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Le Moulin de Champie</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>À 15 min</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Grande maison à louer, à quinze minutes de la ferme.</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>https://www.moulindechampie.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>HÔTELS (environ 10 min en voiture) — pas de description affichée</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>L05</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Hôtels</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Appart'City Versailles Saint-Cyr-l'École</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>https://www.appartcity.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>L06</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Hôtels</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Best Western Paris Saint-Quentin</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>https://www.bestwestern.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>L07</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Hôtels</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Hôtel B&amp;B Rocquencourt</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>https://www.hotel-bb.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>L08</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Hôtels</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Hôtel Première Classe Versailles Saint-Cyr-l'École</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>https://www.premiereclasse.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>L09</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Hôtels</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Ibis Budget Versailles Château Saint-Cyr</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>https://www.accorhotels.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>L10</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Hôtels</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>La Clémencerie</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>https://www.chambres-hotes.fr</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2136,7 +2662,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Embed the Tally RSVP form in the response section
Replaces the placeholder button with the form itself, so guests answer
without leaving the page. Transparent background and hidden title let it
sit inside the existing white card; dynamicHeight lets Tally resize the
iframe as conditional questions appear.

Keeps the public /r/ link as a text fallback underneath, for browsers
that block third-party iframes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -727,12 +727,12 @@
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>P01</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Noms du couple</t>
         </is>
@@ -744,12 +744,12 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>P02</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Date affichée</t>
         </is>
@@ -761,12 +761,12 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>P03</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Début de l'événement (agenda)</t>
         </is>
@@ -778,12 +778,12 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>P04</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Fin de l'événement (agenda)</t>
         </is>
@@ -795,12 +795,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>P05</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Nom du lieu</t>
         </is>
@@ -812,12 +812,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>P06</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Adresse du lieu</t>
         </is>
@@ -829,12 +829,12 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>P07</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Recherche Google Maps</t>
         </is>
@@ -846,12 +846,12 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>P08</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Date limite de réponse</t>
         </is>
@@ -863,25 +863,29 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>P09</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Lien du formulaire RSVP</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr"/>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>https://tally.so/r/XxXDbP</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Lien de la cagnotte</t>
         </is>
@@ -934,12 +938,12 @@
       <c r="C2" s="7" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>A01</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -951,12 +955,12 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>A02</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Noms</t>
         </is>
@@ -968,12 +972,12 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>A03</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -985,12 +989,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>A04</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Lieu</t>
         </is>
@@ -1002,12 +1006,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>A05</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Invitation à défiler</t>
         </is>
@@ -1028,12 +1032,12 @@
       <c r="C8" s="7" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>A06</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Paragraphe</t>
         </is>
@@ -1045,12 +1049,12 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>A07</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -1071,12 +1075,12 @@
       <c r="C11" s="7" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>A08</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1088,12 +1092,12 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>A09</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1105,12 +1109,12 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>A10</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -1122,12 +1126,12 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>A11</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Étiquette 1</t>
         </is>
@@ -1139,12 +1143,12 @@
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>A12</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Étiquette 2</t>
         </is>
@@ -1156,12 +1160,12 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>A13</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Étiquette 3</t>
         </is>
@@ -1173,12 +1177,12 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>A14</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Étiquette 4</t>
         </is>
@@ -1190,12 +1194,12 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>A15</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Lien agenda</t>
         </is>
@@ -1216,12 +1220,12 @@
       <c r="C20" s="7" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>A16</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1233,12 +1237,12 @@
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>A17</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1250,12 +1254,12 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>A18</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Carte 1 — titre</t>
         </is>
@@ -1267,12 +1271,12 @@
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>A19</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Carte 1 — lien</t>
         </is>
@@ -1284,12 +1288,12 @@
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>A20</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Carte 2 — titre</t>
         </is>
@@ -1301,12 +1305,12 @@
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>A21</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Carte 2 — texte</t>
         </is>
@@ -1318,12 +1322,12 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>A22</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Carte 3 — titre</t>
         </is>
@@ -1335,12 +1339,12 @@
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>A23</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Carte 3 — texte</t>
         </is>
@@ -1352,12 +1356,12 @@
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>A24</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Carte 4 — titre</t>
         </is>
@@ -1369,12 +1373,12 @@
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>A25</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Carte 4 — texte</t>
         </is>
@@ -1506,12 +1510,12 @@
       <c r="C38" s="7" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>A32</t>
         </is>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1523,12 +1527,12 @@
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>A33</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1540,12 +1544,12 @@
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>A34</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="9" t="inlineStr">
         <is>
           <t>Texte</t>
         </is>
@@ -1557,29 +1561,29 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="A42" s="9" t="inlineStr">
         <is>
           <t>A35</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>Bouton</t>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Lien de secours (si le formulaire ne charge pas)</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Je confirme ma présence</t>
+          <t>Ouvrez-le dans un nouvel onglet →</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>A36</t>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
         <is>
           <t>Date limite</t>
         </is>
@@ -1600,12 +1604,12 @@
       <c r="C44" s="7" t="n"/>
     </row>
     <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>A37</t>
         </is>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1617,12 +1621,12 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="A46" s="9" t="inlineStr">
         <is>
           <t>A38</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B46" s="9" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1634,12 +1638,12 @@
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>A39</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
         <is>
           <t>Texte</t>
         </is>
@@ -1651,12 +1655,12 @@
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="A48" s="9" t="inlineStr">
         <is>
           <t>A40</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -1677,12 +1681,12 @@
       <c r="C49" s="7" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="A50" s="9" t="inlineStr">
         <is>
           <t>A41</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>Signature</t>
         </is>
@@ -1694,12 +1698,12 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="A51" s="9" t="inlineStr">
         <is>
           <t>A42</t>
         </is>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B51" s="9" t="inlineStr">
         <is>
           <t>Petite phrase</t>
         </is>
@@ -1711,12 +1715,12 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="A52" s="9" t="inlineStr">
         <is>
           <t>A43</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B52" s="9" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -1737,12 +1741,12 @@
       <c r="C53" s="7" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="A54" s="9" t="inlineStr">
         <is>
           <t>A44</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B54" s="9" t="inlineStr">
         <is>
           <t>Titre de l'onglet</t>
         </is>
@@ -1754,12 +1758,12 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="A55" s="9" t="inlineStr">
         <is>
           <t>A45</t>
         </is>
       </c>
-      <c r="B55" s="8" t="inlineStr">
+      <c r="B55" s="9" t="inlineStr">
         <is>
           <t>Description au partage</t>
         </is>
@@ -2196,12 +2200,12 @@
       <c r="C2" s="7" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>H01</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Lien retour</t>
         </is>
@@ -2213,12 +2217,12 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>H02</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Lien raccourci</t>
         </is>
@@ -2239,12 +2243,12 @@
       <c r="C5" s="7" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>H03</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -2256,12 +2260,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>H04</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -2273,12 +2277,12 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>H05</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -2299,12 +2303,12 @@
       <c r="C9" s="7" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>H06</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -2316,12 +2320,12 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>H07</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -2333,12 +2337,12 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>H08</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -2350,12 +2354,12 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>H09</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Étiquette album 1</t>
         </is>
@@ -2367,12 +2371,12 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>H10</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Étiquette album 2</t>
         </is>
@@ -2393,12 +2397,12 @@
       <c r="C15" s="7" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>H11</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -2410,12 +2414,12 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>H12</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -2427,12 +2431,12 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>H13</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -2444,12 +2448,12 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>H14</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Étiquette album 1</t>
         </is>
@@ -2461,12 +2465,12 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>H15</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Étiquette album 2</t>
         </is>
@@ -2487,12 +2491,12 @@
       <c r="C21" s="7" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>H16</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -2504,12 +2508,12 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>H17</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -2521,12 +2525,12 @@
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>H18</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -2547,12 +2551,12 @@
       <c r="C25" s="7" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>H19</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -2564,12 +2568,12 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>H20</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Phrase de fin</t>
         </is>
@@ -2581,12 +2585,12 @@
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>H21</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Texte</t>
         </is>
@@ -2598,12 +2602,12 @@
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>H22</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -2624,12 +2628,12 @@
       <c r="C30" s="7" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>H23</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>Titre de l'onglet</t>
         </is>
@@ -2641,12 +2645,12 @@
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>H24</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Description au partage</t>
         </is>
@@ -2717,12 +2721,12 @@
       <c r="E2" s="7" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>F01</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Ouverture</t>
         </is>
@@ -2730,7 +2734,7 @@
       <c r="C3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>histoire-01-ouverture.jpg</t>
         </is>
@@ -2753,12 +2757,12 @@
       <c r="E4" s="7" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>F02</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2766,7 +2770,7 @@
       <c r="C5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-1.jpg</t>
         </is>
@@ -2778,12 +2782,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>F03</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2791,7 +2795,7 @@
       <c r="C6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-2.jpg</t>
         </is>
@@ -2803,12 +2807,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>F04</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2816,7 +2820,7 @@
       <c r="C7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-3.jpg</t>
         </is>
@@ -2828,12 +2832,12 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>F05</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2841,7 +2845,7 @@
       <c r="C8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-4.jpg</t>
         </is>
@@ -2853,12 +2857,12 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>F06</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2866,7 +2870,7 @@
       <c r="C9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-5.jpg</t>
         </is>
@@ -2878,12 +2882,12 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>F07</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2891,7 +2895,7 @@
       <c r="C10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-6.jpg</t>
         </is>
@@ -2914,12 +2918,12 @@
       <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>F08</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -2927,7 +2931,7 @@
       <c r="C12" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-1.jpg</t>
         </is>
@@ -2939,12 +2943,12 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>F09</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -2952,7 +2956,7 @@
       <c r="C13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-2.jpg</t>
         </is>
@@ -2964,12 +2968,12 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>F10</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -2977,7 +2981,7 @@
       <c r="C14" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-3.jpg</t>
         </is>
@@ -2989,12 +2993,12 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>F11</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -3002,7 +3006,7 @@
       <c r="C15" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-4.jpg</t>
         </is>
@@ -3025,12 +3029,12 @@
       <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>F12</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3038,7 +3042,7 @@
       <c r="C17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-1.jpg</t>
         </is>
@@ -3050,12 +3054,12 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>F13</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3063,7 +3067,7 @@
       <c r="C18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-2.jpg</t>
         </is>
@@ -3075,12 +3079,12 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>F14</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3088,7 +3092,7 @@
       <c r="C19" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-3.jpg</t>
         </is>
@@ -3100,12 +3104,12 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>F15</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3113,7 +3117,7 @@
       <c r="C20" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-4.jpg</t>
         </is>
@@ -3125,12 +3129,12 @@
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>F16</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3138,7 +3142,7 @@
       <c r="C21" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-5.jpg</t>
         </is>
@@ -3150,12 +3154,12 @@
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>F17</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3163,7 +3167,7 @@
       <c r="C22" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-6.jpg</t>
         </is>
@@ -3186,12 +3190,12 @@
       <c r="E23" s="7" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>F18</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3199,7 +3203,7 @@
       <c r="C24" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-1.jpg</t>
         </is>
@@ -3211,12 +3215,12 @@
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>F19</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3224,7 +3228,7 @@
       <c r="C25" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-2.jpg</t>
         </is>
@@ -3236,12 +3240,12 @@
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>F20</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3249,7 +3253,7 @@
       <c r="C26" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-3.jpg</t>
         </is>
@@ -3261,12 +3265,12 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>F21</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3274,7 +3278,7 @@
       <c r="C27" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-4.jpg</t>
         </is>
@@ -3286,12 +3290,12 @@
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>F22</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3299,7 +3303,7 @@
       <c r="C28" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-5.jpg</t>
         </is>
@@ -3311,12 +3315,12 @@
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>F23</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3324,7 +3328,7 @@
       <c r="C29" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D29" s="8" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-6.jpg</t>
         </is>
@@ -3347,12 +3351,12 @@
       <c r="E30" s="7" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>F24</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -3360,7 +3364,7 @@
       <c r="C31" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D31" s="8" t="inlineStr">
+      <c r="D31" s="9" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-1.jpg</t>
         </is>
@@ -3368,12 +3372,12 @@
       <c r="E31" s="6" t="inlineStr"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>F25</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -3381,7 +3385,7 @@
       <c r="C32" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D32" s="8" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-2.jpg</t>
         </is>
@@ -3389,12 +3393,12 @@
       <c r="E32" s="6" t="inlineStr"/>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>F26</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -3402,7 +3406,7 @@
       <c r="C33" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D33" s="8" t="inlineStr">
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-3.jpg</t>
         </is>
@@ -3410,12 +3414,12 @@
       <c r="E33" s="6" t="inlineStr"/>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>F27</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -3423,7 +3427,7 @@
       <c r="C34" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-4.jpg</t>
         </is>
@@ -3431,12 +3435,12 @@
       <c r="E34" s="6" t="inlineStr"/>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>F28</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -3444,7 +3448,7 @@
       <c r="C35" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D35" s="8" t="inlineStr">
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-5.jpg</t>
         </is>
@@ -3463,12 +3467,12 @@
       <c r="E36" s="7" t="n"/>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>F29</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>Épilogue</t>
         </is>
@@ -3476,7 +3480,7 @@
       <c r="C37" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="8" t="inlineStr">
+      <c r="D37" s="9" t="inlineStr">
         <is>
           <t>histoire-07-epilogue.jpg</t>
         </is>

</xml_diff>

<commit_message>
Activate the gift-pot button with the OnParticipe link
Uses the site's own primary button rather than OnParticipe's supplied
snippet, whose inline styles (black 2px borders, Inter, fixed 224px
width) would not survive next to the pastel palette and would overflow
narrow phones.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -890,7 +890,11 @@
           <t>Lien de la cagnotte</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr"/>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>https://www.onparticipe.fr/c/GsV9G6xD</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1667,7 +1671,7 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Accéder à la cagnotte</t>
+          <t>Je participe →</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
New cover photo, rework chapter III, link hotels directly
Swaps the hero for "photo accueil new" and nudges object-position to 20%
so the faces clear the crop on wide screens.

Chapter III drops the terrace selfie, which duplicated the Calanques one
(same summer close-up, both in sunglasses). The Calanques frame is
re-cropped to 3:4 from the original 2048x1536 rather than being
center-cropped by object-fit, which was cutting one of them out. Adds
the red-dress and horseback photos, taking the deck to six.

Hotel entries now deep-link to each property instead of the chain
homepage. Two notes:
- the Saint-Cyr Appart'City is now a Comfort Aparthotel (Zenitude) at
  the same address, so the name is updated
- bestwestern.fr and premiereclasse.com return 403 to automated
  requests, so those two URLs are unverified

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -141,6 +141,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -727,12 +736,12 @@
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>P01</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Noms du couple</t>
         </is>
@@ -744,12 +753,12 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>P02</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Date affichée</t>
         </is>
@@ -761,12 +770,12 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>P03</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Début de l'événement (agenda)</t>
         </is>
@@ -778,12 +787,12 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>P04</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Fin de l'événement (agenda)</t>
         </is>
@@ -795,12 +804,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>P05</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Nom du lieu</t>
         </is>
@@ -812,12 +821,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>P06</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Adresse du lieu</t>
         </is>
@@ -829,12 +838,12 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>P07</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Recherche Google Maps</t>
         </is>
@@ -846,12 +855,12 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>P08</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Date limite de réponse</t>
         </is>
@@ -863,12 +872,12 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>P09</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Lien du formulaire RSVP</t>
         </is>
@@ -880,12 +889,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Lien de la cagnotte</t>
         </is>
@@ -942,12 +951,12 @@
       <c r="C2" s="7" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>A01</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -959,12 +968,12 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>A02</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Noms</t>
         </is>
@@ -976,12 +985,12 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>A03</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -993,12 +1002,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>A04</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Lieu</t>
         </is>
@@ -1010,12 +1019,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>A05</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Invitation à défiler</t>
         </is>
@@ -1036,12 +1045,12 @@
       <c r="C8" s="7" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>A06</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Paragraphe</t>
         </is>
@@ -1053,12 +1062,12 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>A07</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -1079,12 +1088,12 @@
       <c r="C11" s="7" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>A08</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1096,12 +1105,12 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>A09</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1113,12 +1122,12 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>A10</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -1130,12 +1139,12 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>A11</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Étiquette 1</t>
         </is>
@@ -1147,12 +1156,12 @@
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>A12</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Étiquette 2</t>
         </is>
@@ -1164,12 +1173,12 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>A13</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Étiquette 3</t>
         </is>
@@ -1181,12 +1190,12 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>A14</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Étiquette 4</t>
         </is>
@@ -1198,12 +1207,12 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>A15</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Lien agenda</t>
         </is>
@@ -1224,12 +1233,12 @@
       <c r="C20" s="7" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>A16</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1241,12 +1250,12 @@
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>A17</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1258,12 +1267,12 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>A18</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Carte 1 — titre</t>
         </is>
@@ -1275,12 +1284,12 @@
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>A19</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Carte 1 — lien</t>
         </is>
@@ -1292,12 +1301,12 @@
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>A20</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Carte 2 — titre</t>
         </is>
@@ -1309,12 +1318,12 @@
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>A21</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Carte 2 — texte</t>
         </is>
@@ -1326,12 +1335,12 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>A22</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Carte 3 — titre</t>
         </is>
@@ -1343,12 +1352,12 @@
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>A23</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Carte 3 — texte</t>
         </is>
@@ -1360,12 +1369,12 @@
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>A24</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Carte 4 — titre</t>
         </is>
@@ -1377,12 +1386,12 @@
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>A25</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>Carte 4 — texte</t>
         </is>
@@ -1403,12 +1412,12 @@
       <c r="C31" s="7" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>A26</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1420,12 +1429,12 @@
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="9" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>A27</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1437,12 +1446,12 @@
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>A28</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>Texte d'introduction</t>
         </is>
@@ -1454,12 +1463,12 @@
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>A29</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>Titre du groupe 1</t>
         </is>
@@ -1471,12 +1480,12 @@
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>Titre du groupe 2</t>
         </is>
@@ -1488,12 +1497,12 @@
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="9" t="inlineStr">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>A31</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>Sous-titre groupe 2</t>
         </is>
@@ -1514,12 +1523,12 @@
       <c r="C38" s="7" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="9" t="inlineStr">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>A32</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1531,12 +1540,12 @@
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="9" t="inlineStr">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>A33</t>
         </is>
       </c>
-      <c r="B40" s="9" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1548,12 +1557,12 @@
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="9" t="inlineStr">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>A34</t>
         </is>
       </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>Texte</t>
         </is>
@@ -1565,12 +1574,12 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>A35</t>
         </is>
       </c>
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B42" s="11" t="inlineStr">
         <is>
           <t>Lien de secours (si le formulaire ne charge pas)</t>
         </is>
@@ -1582,12 +1591,12 @@
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="9" t="inlineStr">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>A36</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>Date limite</t>
         </is>
@@ -1608,12 +1617,12 @@
       <c r="C44" s="7" t="n"/>
     </row>
     <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="9" t="inlineStr">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>A37</t>
         </is>
       </c>
-      <c r="B45" s="9" t="inlineStr">
+      <c r="B45" s="11" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -1625,12 +1634,12 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="inlineStr">
+      <c r="A46" s="11" t="inlineStr">
         <is>
           <t>A38</t>
         </is>
       </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="B46" s="11" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -1642,12 +1651,12 @@
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="9" t="inlineStr">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t>A39</t>
         </is>
       </c>
-      <c r="B47" s="9" t="inlineStr">
+      <c r="B47" s="11" t="inlineStr">
         <is>
           <t>Texte</t>
         </is>
@@ -1659,12 +1668,12 @@
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="9" t="inlineStr">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t>A40</t>
         </is>
       </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="B48" s="11" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -1685,12 +1694,12 @@
       <c r="C49" s="7" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="9" t="inlineStr">
+      <c r="A50" s="11" t="inlineStr">
         <is>
           <t>A41</t>
         </is>
       </c>
-      <c r="B50" s="9" t="inlineStr">
+      <c r="B50" s="11" t="inlineStr">
         <is>
           <t>Signature</t>
         </is>
@@ -1702,12 +1711,12 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>A42</t>
         </is>
       </c>
-      <c r="B51" s="9" t="inlineStr">
+      <c r="B51" s="11" t="inlineStr">
         <is>
           <t>Petite phrase</t>
         </is>
@@ -1719,12 +1728,12 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="inlineStr">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>A43</t>
         </is>
       </c>
-      <c r="B52" s="9" t="inlineStr">
+      <c r="B52" s="11" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -1745,12 +1754,12 @@
       <c r="C53" s="7" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="9" t="inlineStr">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t>A44</t>
         </is>
       </c>
-      <c r="B54" s="9" t="inlineStr">
+      <c r="B54" s="11" t="inlineStr">
         <is>
           <t>Titre de l'onglet</t>
         </is>
@@ -1762,12 +1771,12 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="9" t="inlineStr">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t>A45</t>
         </is>
       </c>
-      <c r="B55" s="9" t="inlineStr">
+      <c r="B55" s="11" t="inlineStr">
         <is>
           <t>Description au partage</t>
         </is>
@@ -1852,17 +1861,17 @@
       <c r="G2" s="7" t="n"/>
     </row>
     <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>L01</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Gîtes et maisons</t>
         </is>
       </c>
-      <c r="C3" s="10" t="n">
+      <c r="C3" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -1870,7 +1879,7 @@
           <t>Le Gîte de la Ferme de Pontaly</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>À 10 min</t>
         </is>
@@ -1880,24 +1889,24 @@
           <t>Une véritable ferme agricole spécialisée en grandes cultures bio. Elle possède 3 gîtes, de 4 à 8 personnes.</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="G3" s="12" t="inlineStr">
         <is>
           <t>https://www.fermedepontaly.fr</t>
         </is>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>L02</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Gîtes et maisons</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -1905,7 +1914,7 @@
           <t>La Ferme de Mezu</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>À 5 min</t>
         </is>
@@ -1915,20 +1924,20 @@
           <t>Jolie ferme équestre et céréalière à Chavenay, en plein milieu des champs. 2 gîtes ruraux (4 et 6 personnes). Réservation sur Gîtes de France.</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr"/>
+      <c r="G4" s="12" t="inlineStr"/>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>L03</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Gîtes et maisons</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="12" t="n">
         <v>3</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1936,30 +1945,30 @@
           <t>Le Val Trebbia</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr"/>
+      <c r="E5" s="12" t="inlineStr"/>
       <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Maison d'hôtes située à Feucherolles.</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t>https://val-trebbia.fr</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>L04</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Gîtes et maisons</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="12" t="n">
         <v>4</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1967,7 +1976,7 @@
           <t>Le Moulin de Champie</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>À 15 min</t>
         </is>
@@ -1977,7 +1986,7 @@
           <t>Grande maison à louer, à quinze minutes de la ferme.</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>https://www.moulindechampie.com</t>
         </is>
@@ -1997,44 +2006,44 @@
       <c r="G7" s="7" t="n"/>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>L05</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Hôtels</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Appart'City Versailles Saint-Cyr-l'École</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr"/>
+          <t>Comfort Aparthotel Versailles Saint-Cyr-l'École</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr"/>
       <c r="F8" s="6" t="inlineStr"/>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>https://www.appartcity.com</t>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>https://www.zenitude-hotel-residences.com/residences/versailles-st-cyr-lecole/</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>L06</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Hôtels</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -2042,107 +2051,107 @@
           <t>Best Western Paris Saint-Quentin</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr"/>
+      <c r="E9" s="12" t="inlineStr"/>
       <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>https://www.bestwestern.fr</t>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>https://www.bestwestern.fr/fr/hotel-Montigny-Le-Bretonneux-BEST-WESTERN-Paris-Saint-Quentin-93842</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>L07</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Hôtels</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="12" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Hôtel B&amp;B Rocquencourt</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr"/>
+          <t>B&amp;B Hôtel Versailles Rocquencourt</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr"/>
       <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>https://www.hotel-bb.com</t>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>https://www.hotel-bb.com/fr/hotel/versailles-rocquencourt</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>L08</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Hôtels</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="12" t="n">
         <v>4</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Hôtel Première Classe Versailles Saint-Cyr-l'École</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr"/>
+          <t>Première Classe Versailles Saint-Cyr-l'École</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr"/>
       <c r="F11" s="6" t="inlineStr"/>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>https://www.premiereclasse.com</t>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>https://versailles-saint-cyr-lecole.premiereclasse.com/</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>L09</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Hôtels</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="12" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Ibis Budget Versailles Château Saint-Cyr</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr"/>
+          <t>ibis budget Versailles Château Saint-Cyr</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr"/>
       <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>https://www.accorhotels.com</t>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>https://all.accor.com/hotel/2567/index.fr.shtml</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>L10</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Hôtels</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="12" t="n">
         <v>6</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -2150,11 +2159,11 @@
           <t>La Clémencerie</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr"/>
+      <c r="E13" s="12" t="inlineStr"/>
       <c r="F13" s="6" t="inlineStr"/>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>https://www.chambres-hotes.fr</t>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>https://www.chambres-hotes.fr/chambres-hotes_la-clemencerie_l-etang-la-ville_h1379867.htm</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2213,12 @@
       <c r="C2" s="7" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>H01</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Lien retour</t>
         </is>
@@ -2221,12 +2230,12 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>H02</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Lien raccourci</t>
         </is>
@@ -2247,12 +2256,12 @@
       <c r="C5" s="7" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>H03</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Surtitre</t>
         </is>
@@ -2264,12 +2273,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>H04</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -2281,12 +2290,12 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>H05</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -2307,12 +2316,12 @@
       <c r="C9" s="7" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>H06</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -2324,12 +2333,12 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>H07</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -2341,12 +2350,12 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>H08</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -2358,12 +2367,12 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>H09</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Étiquette album 1</t>
         </is>
@@ -2375,12 +2384,12 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>H10</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Étiquette album 2</t>
         </is>
@@ -2401,12 +2410,12 @@
       <c r="C15" s="7" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>H11</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -2418,12 +2427,12 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>H12</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -2435,12 +2444,12 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>H13</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -2452,12 +2461,12 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>H14</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Étiquette album 1</t>
         </is>
@@ -2469,12 +2478,12 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>H15</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Étiquette album 2</t>
         </is>
@@ -2495,12 +2504,12 @@
       <c r="C21" s="7" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>H16</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -2512,12 +2521,12 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>H17</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
@@ -2529,12 +2538,12 @@
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>H18</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Sous-titre</t>
         </is>
@@ -2555,12 +2564,12 @@
       <c r="C25" s="7" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>H19</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -2572,12 +2581,12 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>H20</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Phrase de fin</t>
         </is>
@@ -2589,12 +2598,12 @@
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>H21</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Texte</t>
         </is>
@@ -2606,12 +2615,12 @@
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>H22</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Bouton</t>
         </is>
@@ -2632,12 +2641,12 @@
       <c r="C30" s="7" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>H23</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Titre de l'onglet</t>
         </is>
@@ -2649,12 +2658,12 @@
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>H24</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Description au partage</t>
         </is>
@@ -2676,7 +2685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2725,12 +2734,12 @@
       <c r="E2" s="7" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>F01</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Ouverture</t>
         </is>
@@ -2738,7 +2747,7 @@
       <c r="C3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>histoire-01-ouverture.jpg</t>
         </is>
@@ -2761,12 +2770,12 @@
       <c r="E4" s="7" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>F02</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2774,7 +2783,7 @@
       <c r="C5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-1.jpg</t>
         </is>
@@ -2786,12 +2795,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>F03</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2799,7 +2808,7 @@
       <c r="C6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-2.jpg</t>
         </is>
@@ -2811,12 +2820,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>F04</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2824,7 +2833,7 @@
       <c r="C7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-3.jpg</t>
         </is>
@@ -2836,12 +2845,12 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>F05</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2849,7 +2858,7 @@
       <c r="C8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-4.jpg</t>
         </is>
@@ -2861,12 +2870,12 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>F06</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2874,7 +2883,7 @@
       <c r="C9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-5.jpg</t>
         </is>
@@ -2886,12 +2895,12 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>F07</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Ch. I — Elle</t>
         </is>
@@ -2899,7 +2908,7 @@
       <c r="C10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>histoire-02-ch1-elle-6.jpg</t>
         </is>
@@ -2922,12 +2931,12 @@
       <c r="E11" s="7" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>F08</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -2935,7 +2944,7 @@
       <c r="C12" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-1.jpg</t>
         </is>
@@ -2947,12 +2956,12 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>F09</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -2960,7 +2969,7 @@
       <c r="C13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-2.jpg</t>
         </is>
@@ -2972,12 +2981,12 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>F10</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -2985,7 +2994,7 @@
       <c r="C14" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-3.jpg</t>
         </is>
@@ -2997,12 +3006,12 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>F11</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Ch. I — Lui</t>
         </is>
@@ -3010,7 +3019,7 @@
       <c r="C15" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>histoire-03-ch1-lui-4.jpg</t>
         </is>
@@ -3033,12 +3042,12 @@
       <c r="E16" s="7" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>F12</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3046,7 +3055,7 @@
       <c r="C17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-1.jpg</t>
         </is>
@@ -3058,12 +3067,12 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>F13</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3071,7 +3080,7 @@
       <c r="C18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-2.jpg</t>
         </is>
@@ -3083,12 +3092,12 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>F14</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3096,7 +3105,7 @@
       <c r="C19" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-3.jpg</t>
         </is>
@@ -3108,12 +3117,12 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>F15</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3121,7 +3130,7 @@
       <c r="C20" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-4.jpg</t>
         </is>
@@ -3133,12 +3142,12 @@
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>F16</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3146,7 +3155,7 @@
       <c r="C21" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-5.jpg</t>
         </is>
@@ -3158,12 +3167,12 @@
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>F17</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Elle</t>
         </is>
@@ -3171,7 +3180,7 @@
       <c r="C22" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>histoire-04-ch2-elle-6.jpg</t>
         </is>
@@ -3194,12 +3203,12 @@
       <c r="E23" s="7" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>F18</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3207,7 +3216,7 @@
       <c r="C24" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-1.jpg</t>
         </is>
@@ -3219,12 +3228,12 @@
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>F19</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3232,7 +3241,7 @@
       <c r="C25" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-2.jpg</t>
         </is>
@@ -3244,12 +3253,12 @@
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>F20</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3257,7 +3266,7 @@
       <c r="C26" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-3.jpg</t>
         </is>
@@ -3269,12 +3278,12 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>F21</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3282,7 +3291,7 @@
       <c r="C27" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-4.jpg</t>
         </is>
@@ -3294,12 +3303,12 @@
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>F22</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3307,7 +3316,7 @@
       <c r="C28" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-5.jpg</t>
         </is>
@@ -3319,12 +3328,12 @@
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>F23</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Ch. II — Lui</t>
         </is>
@@ -3332,7 +3341,7 @@
       <c r="C29" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>histoire-05-ch2-lui-6.jpg</t>
         </is>
@@ -3355,12 +3364,12 @@
       <c r="E30" s="7" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>F24</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -3368,7 +3377,7 @@
       <c r="C31" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-1.jpg</t>
         </is>
@@ -3376,12 +3385,12 @@
       <c r="E31" s="6" t="inlineStr"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>F25</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -3389,7 +3398,7 @@
       <c r="C32" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-2.jpg</t>
         </is>
@@ -3397,12 +3406,12 @@
       <c r="E32" s="6" t="inlineStr"/>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="9" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>F26</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -3410,7 +3419,7 @@
       <c r="C33" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-3.jpg</t>
         </is>
@@ -3418,12 +3427,12 @@
       <c r="E33" s="6" t="inlineStr"/>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>F27</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -3431,7 +3440,7 @@
       <c r="C34" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-4.jpg</t>
         </is>
@@ -3439,12 +3448,12 @@
       <c r="E34" s="6" t="inlineStr"/>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>F28</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>Ch. III</t>
         </is>
@@ -3452,44 +3461,65 @@
       <c r="C35" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D35" s="11" t="inlineStr">
         <is>
           <t>histoire-06-ch3-trouves-5.jpg</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr"/>
     </row>
-    <row r="36">
-      <c r="A36" s="7" t="inlineStr">
+    <row r="36" ht="34" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>F29</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Ch. III</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>histoire-06-ch3-trouves-6.jpg</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>ÉPILOGUE</t>
         </is>
       </c>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="9" t="inlineStr">
-        <is>
-          <t>F29</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="7" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>F30</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Épilogue</t>
         </is>
       </c>
-      <c r="C37" s="6" t="n">
+      <c r="C38" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>histoire-07-epilogue.jpg</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>Et depuis, ils ne marchent plus l'un sans l'autre.</t>
         </is>

</xml_diff>

<commit_message>
Realign two spreadsheet cells with the live site
The share description still held the sentence dropped in the rewrite, and
the dress-code line had a comma where the site has a semicolon.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -590,14 +590,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="B2:B34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="20.25" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -746,7 +745,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="16.5" customHeight="1">
       <c r="B27" s="3" t="inlineStr">
         <is>
@@ -775,7 +773,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32" ht="16.5" customHeight="1">
       <c r="B32" s="17" t="inlineStr">
         <is>
@@ -1466,7 +1463,7 @@
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>Chic et simple : costume pour les loups de Wall Street, chemise et chino pour les bg timides, tailleurs, pantalons, jupes, robe pour les audacieuses.</t>
+          <t>Chic et simple : costume pour les loups de Wall Street, chemise et chino pour les bg timides, tailleurs, pantalons, jupes ; robe pour les audacieuses.</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1884,7 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>On se marie à la Ferme de la Faisanderie. On serait ravis de vous avoir à nos côtés.</t>
+          <t>Eh oui, nous nous marions ! Rendez-vous le 24 avril 2027 à la Ferme de la Faisanderie.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sunday is a brunch at 11h30, with galettes and crêpes
Replaces "petit-déjeuner" in both the programme and the table card, adds
the menu, and gives the table card the time it was missing — the two
cards disagreed on the hour before.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -1428,8 +1428,8 @@
           <t>Samedi 24 avril 2027 : 
 Cocktail au milieu des champs à partir de 17h.
 Dîner sous la charpente de la Grange à Grains, et DJ jusqu'au bout de la nuit.
-Dimanche 25 avril 2027: 
-Petit-déjeuner à la ferme, dès 11h00.</t>
+Dimanche 25 avril 2027 : 
+Brunch à la ferme, dès 11h30.</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
         <is>
           <t>Pour commencer, un cocktail en plein air avec des bouchées gourmandes, du champagne, du spritz et les bières de la brasserie Toussaint, brassées à Noisy-le-Roi. Ensuite, le brasero prend le relais avec des grillades au feu de bois à déguster autour d'une grande tablée.
 Il n'y a pas de plan de table : servez-vous quand vous voulez et asseyez-vous où vous voulez.
-Dimanche, un petit-déjeuner attend les rescapés de la veille, parce qu'un vrai hobbit n'en saute jamais un.</t>
+Dimanche, dès 11h30, un brunch attend les rescapés de la veille : galettes bretonnes salées et crêpes sucrées. Parce qu'un vrai hobbit ne saute jamais un repas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split the calendar into two events side by side
One 21-hour block spanning the night was unwieldy in a phone calendar.
Saturday now runs 17h00-03h00 and the brunch 11h30-14h30, as two links
that sit on one line and wrap on narrow screens. Each carries its own
description.

CONFIG gains brunchStartISO/brunchEndISO, and the spreadsheet's
Paramètres tab the matching rows — which shifts the deadline from P08 to
P10, so the cross-reference in the Accueil tab is updated too.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -93,7 +93,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -130,8 +130,18 @@
         <fgColor rgb="FFFFF9D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFE8E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9D6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -169,12 +179,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D8CCC4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D8CCC4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D8CCC4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D8CCC4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,6 +247,15 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -805,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -872,7 +905,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Début de l'événement (agenda)</t>
+          <t>Samedi — début (agenda)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -889,46 +922,46 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Fin de l'événement (agenda)</t>
+          <t>Samedi — fin (agenda)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>2027-04-25T14:00:00</t>
+          <t>2027-04-25T03:00:00</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>P05</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Nom du lieu</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>La Ferme de la Faisanderie</t>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Brunch dimanche — début (agenda)</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>2027-04-25T11:30:00</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>P06</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Adresse du lieu</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Route de Rennemoulin, 78450 Villepreux</t>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Brunch dimanche — fin (agenda)</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>2027-04-25T14:30:00</t>
         </is>
       </c>
     </row>
@@ -940,12 +973,12 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Recherche Google Maps</t>
+          <t>Nom du lieu</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Ferme de la Faisanderie, Route de Rennemoulin, 78450 Villepreux</t>
+          <t>La Ferme de la Faisanderie</t>
         </is>
       </c>
     </row>
@@ -957,12 +990,12 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Date limite de réponse</t>
+          <t>Adresse du lieu</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>1er février 2027</t>
+          <t>Route de Rennemoulin, 78450 Villepreux</t>
         </is>
       </c>
     </row>
@@ -974,12 +1007,12 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Lien du formulaire RSVP</t>
+          <t>Recherche Google Maps</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>https://tally.so/r/XxXDbP</t>
+          <t>Ferme de la Faisanderie, Route de Rennemoulin, 78450 Villepreux</t>
         </is>
       </c>
     </row>
@@ -991,10 +1024,44 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
+          <t>Date limite de réponse</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>1er février 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Lien du formulaire RSVP</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>https://tally.so/r/XxXDbP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
           <t>Lien de la cagnotte</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>https://www.onparticipe.fr/c/GsV9G6xD</t>
         </is>
@@ -1011,7 +1078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1309,40 +1376,40 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Lien agenda</t>
+          <t>Lien agenda — samedi</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+ Ajouter à mon calendrier</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+          <t>+ Ajouter le samedi</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>A16</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>Lien agenda — brunch</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>+ Ajouter le brunch</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>INFOS PRATIQUES</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>A16</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Surtitre</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Bon à savoir</t>
-        </is>
-      </c>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -1352,12 +1419,12 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Titre</t>
+          <t>Surtitre</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Infos pratiques</t>
+          <t>Bon à savoir</t>
         </is>
       </c>
     </row>
@@ -1369,12 +1436,12 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Carte 1 — titre</t>
+          <t>Titre</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Le lieu</t>
+          <t>Infos pratiques</t>
         </is>
       </c>
     </row>
@@ -1386,12 +1453,12 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Carte 1 — lien</t>
+          <t>Carte 1 — titre</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Voir l'itinéraire →</t>
+          <t>Le lieu</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1470,12 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Carte 2 — titre</t>
+          <t>Carte 1 — lien</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Le programme</t>
+          <t>Voir l'itinéraire →</t>
         </is>
       </c>
     </row>
@@ -1420,10 +1487,27 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
+          <t>Carte 2 — titre</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Le programme</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>A22</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
           <t>Carte 2 — texte</t>
         </is>
       </c>
-      <c r="C26" s="20" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>Samedi 24 avril 2027 : 
 Cocktail au milieu des champs à partir de 17h.
@@ -1433,23 +1517,6 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>A22</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Carte 3 — titre</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>La tenue</t>
-        </is>
-      </c>
-    </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
@@ -1458,12 +1525,12 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Carte 3 — texte</t>
-        </is>
-      </c>
-      <c r="C28" s="20" t="inlineStr">
-        <is>
-          <t>Chic et simple : costume pour les loups de Wall Street, chemise et chino pour les bg timides, tailleurs, pantalons, jupes ; robe pour les audacieuses.</t>
+          <t>Carte 3 — titre</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>La tenue</t>
         </is>
       </c>
     </row>
@@ -1475,12 +1542,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Carte 4 — titre</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>À table</t>
+          <t>Carte 3 — texte</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>Chic et simple : costume pour les loups de Wall Street, chemise et chino pour les bg timides, tailleurs, pantalons, jupes ; robe pour les audacieuses.</t>
         </is>
       </c>
     </row>
@@ -1492,10 +1559,27 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
+          <t>Carte 4 — titre</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>À table</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>A26</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
           <t>Carte 4 — texte</t>
         </is>
       </c>
-      <c r="C30" s="20" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>Pour commencer, un cocktail en plein air avec des bouchées gourmandes, du champagne, du spritz et les bières de la brasserie Toussaint, brassées à Noisy-le-Roi. Ensuite, le brasero prend le relais avec des grillades au feu de bois à déguster autour d'une grande tablée.
 Il n'y a pas de plan de table : servez-vous quand vous voulez et asseyez-vous où vous voulez.
@@ -1503,31 +1587,14 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>HÉBERGEMENTS</t>
         </is>
       </c>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="6" t="n"/>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>A26</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Surtitre</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Où dormir</t>
-        </is>
-      </c>
+      <c r="B32" s="6" t="n"/>
+      <c r="C32" s="6" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
@@ -1537,12 +1604,12 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Titre</t>
+          <t>Surtitre</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Hébergements</t>
+          <t>Où dormir</t>
         </is>
       </c>
     </row>
@@ -1554,12 +1621,12 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Texte d'introduction</t>
+          <t>Titre</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Quelques adresses repérées autour de la ferme. Pensez à réserver tôt, le Poney Fringant n'est déjà plus dispo !</t>
+          <t>Hébergements</t>
         </is>
       </c>
     </row>
@@ -1571,12 +1638,12 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Titre du groupe 1</t>
+          <t>Texte d'introduction</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Gîtes et maisons</t>
+          <t>Quelques adresses repérées autour de la ferme. Pensez à réserver tôt, le Poney Fringant n'est déjà plus dispo !</t>
         </is>
       </c>
     </row>
@@ -1588,12 +1655,12 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Titre du groupe 2</t>
+          <t>Titre du groupe 1</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Hôtels</t>
+          <t>Gîtes et maisons</t>
         </is>
       </c>
     </row>
@@ -1605,40 +1672,40 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
+          <t>Titre du groupe 2</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Hôtels</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>A32</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
           <t>Sous-titre groupe 2</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>Un peu plus éloigné, environ 10 min en voiture</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="6" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>RÉPONSE (RSVP)</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="6" t="n"/>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>A32</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Surtitre</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Votre réponse</t>
-        </is>
-      </c>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="6" t="n"/>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
@@ -1648,12 +1715,12 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Titre</t>
+          <t>Surtitre</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Serez-vous des nôtres ?</t>
+          <t>Votre réponse</t>
         </is>
       </c>
     </row>
@@ -1665,12 +1732,12 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Texte</t>
+          <t>Titre</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Un petit clic pour nous confirmer votre présence : ça nous aide énormément pour l'organisation.</t>
+          <t>Serez-vous des nôtres ?</t>
         </is>
       </c>
     </row>
@@ -1682,12 +1749,12 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Lien de secours (si le formulaire ne charge pas)</t>
+          <t>Texte</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Ouvrez-le dans un nouvel onglet →</t>
+          <t>Un petit clic pour nous confirmer votre présence : ça nous aide énormément pour l'organisation.</t>
         </is>
       </c>
     </row>
@@ -1699,40 +1766,40 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
+          <t>Lien de secours (si le formulaire ne charge pas)</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Ouvrez-le dans un nouvel onglet →</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>A37</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
           <t>Date limite</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Merci de répondre avant le [date — voir onglet Paramètres (P08)]</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Merci de répondre avant le [date — voir onglet Paramètres (P10)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>CAGNOTTE</t>
         </is>
       </c>
-      <c r="B44" s="6" t="n"/>
-      <c r="C44" s="6" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>A37</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>Surtitre</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>Pour nous gâter</t>
-        </is>
-      </c>
+      <c r="B45" s="6" t="n"/>
+      <c r="C45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -1742,12 +1809,12 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Titre</t>
+          <t>Surtitre</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Une cagnotte plutôt que des cadeaux</t>
+          <t>Pour nous gâter</t>
         </is>
       </c>
     </row>
@@ -1759,12 +1826,12 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Texte</t>
-        </is>
-      </c>
-      <c r="C47" s="20" t="inlineStr">
-        <is>
-          <t>Votre présence est évidemment le plus beau des cadeaux ! Si vous souhaitez tout de même nous offrir quelque chose, une participation à notre lune de miel nous ferait plaisir. Une cagnotte est ouverte.</t>
+          <t>Titre</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Une cagnotte plutôt que des cadeaux</t>
         </is>
       </c>
     </row>
@@ -1776,40 +1843,40 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
+          <t>Texte</t>
+        </is>
+      </c>
+      <c r="C48" s="20" t="inlineStr">
+        <is>
+          <t>Votre présence est évidemment le plus beau des cadeaux ! Si vous souhaitez tout de même nous offrir quelque chose, une participation à notre lune de miel nous ferait plaisir. Une cagnotte est ouverte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>A41</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
           <t>Bouton</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Je participe →</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>PIED DE PAGE</t>
         </is>
       </c>
-      <c r="B49" s="6" t="n"/>
-      <c r="C49" s="6" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>A41</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>→ voir onglet Paramètres (P01)</t>
-        </is>
-      </c>
+      <c r="B50" s="6" t="n"/>
+      <c r="C50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -1819,12 +1886,12 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Petite phrase</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Avec impatience de vous voir tous réunis.</t>
+          <t>→ voir onglet Paramètres (P01)</t>
         </is>
       </c>
     </row>
@@ -1836,40 +1903,40 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
+          <t>Petite phrase</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Avec impatience de vous voir tous réunis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>A44</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
           <t>Bouton</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Notre histoire →</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>PARTAGE (aperçu WhatsApp / réseaux)</t>
         </is>
       </c>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>A44</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>Titre de l'onglet</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>Awéna &amp; Grégoire - 24 avril 2027</t>
-        </is>
-      </c>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -1879,10 +1946,27 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
+          <t>Titre de l'onglet</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Awéna &amp; Grégoire - 24 avril 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>A46</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
           <t>Description au partage</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>Eh oui, nous nous marions ! Rendez-vous le 24 avril 2027 à la Ferme de la Faisanderie.</t>
         </is>

</xml_diff>

<commit_message>
Add Le Bout du Parc, drop Le Moulin de Champie
Le Bout du Parc is a hotel, so it goes at the head of the hotels list
rather than in the gîtes grid, which now holds three cards.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -198,7 +198,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -256,6 +256,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -932,12 +941,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>P05</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Brunch dimanche — début (agenda)</t>
         </is>
@@ -949,12 +958,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>P06</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>Brunch dimanche — fin (agenda)</t>
         </is>
@@ -2143,52 +2152,44 @@
       </c>
     </row>
     <row r="6" ht="33.95" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>HÔTELS (environ 10 min en voiture) — pas de description affichée</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>L04</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Gîtes et maisons</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Le Moulin de Champie</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>À 15 min</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Grande maison à louer, à quinze minutes de la ferme.</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>https://www.moulindechampie.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>HÔTELS (environ 10 min en voiture) — pas de description affichée</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Hôtels</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Café-Hôtel Le Bout du Parc</t>
+        </is>
+      </c>
+      <c r="E7" s="25" t="inlineStr"/>
+      <c r="F7" s="22" t="inlineStr"/>
+      <c r="G7" s="25" t="inlineStr">
+        <is>
+          <t>https://www.hotel-boutduparc.com/</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="33.95" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -2202,7 +2203,7 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
@@ -2229,7 +2230,7 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
@@ -2256,7 +2257,7 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
@@ -2283,7 +2284,7 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
@@ -2310,7 +2311,7 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
@@ -2337,7 +2338,7 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
@@ -2364,7 +2365,7 @@
         </is>
       </c>
       <c r="C14" s="11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Say 15 minutes for the hotels group
Le Bout du Parc and La Clémencerie both sit beyond the 10 minutes the
subtitle claimed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -941,12 +941,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>P05</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Brunch dimanche — début (agenda)</t>
         </is>
@@ -958,12 +958,12 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>P06</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Brunch dimanche — fin (agenda)</t>
         </is>
@@ -1395,12 +1395,12 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="23" t="inlineStr">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>A16</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>Lien agenda — brunch</t>
         </is>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Un peu plus éloigné, environ 10 min en voiture</t>
+          <t>Un peu plus éloigné, environ 15 min en voiture</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop Première Classe and ibis budget from the hotels list
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textes-site.xlsx
+++ b/textes-site.xlsx
@@ -1992,7 +1992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2288,102 +2288,50 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Première Classe Versailles Saint-Cyr-l'École</t>
+          <t>La Clémencerie</t>
         </is>
       </c>
       <c r="E11" s="8" t="n"/>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>https://versailles-saint-cyr-lecole.premiereclasse.com/</t>
+          <t>https://www.chambres-hotes.fr/chambres-hotes_la-clemencerie_l-etang-la-ville_h1379867.htm</t>
         </is>
       </c>
     </row>
     <row r="12" ht="33.95" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>L09</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Hôtels</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>ibis budget Versailles Château Saint-Cyr</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>https://all.accor.com/hotel/2567/index.fr.shtml</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="33.95" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>L10</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Hôtels</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>La Clémencerie</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>https://www.chambres-hotes.fr/chambres-hotes_la-clemencerie_l-etang-la-ville_h1379867.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="33.95" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>L11</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Hôtels 5 étoiles</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Chez les parents</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Pour les locaux de l'étape</t>
         </is>
       </c>
-      <c r="F14" s="12" t="inlineStr">
+      <c r="F12" s="12" t="inlineStr">
         <is>
           <t>On y est toujours bien.</t>
         </is>
       </c>
-      <c r="G14" s="19" t="n"/>
-    </row>
+      <c r="G12" s="19" t="n"/>
+    </row>
+    <row r="13" ht="33.95" customHeight="1"/>
+    <row r="14" ht="33.95" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>